<commit_message>
code push for grocery application
</commit_message>
<xml_diff>
--- a/GroceryApplication/src/test/resources/TestingCredentials.xlsx
+++ b/GroceryApplication/src/test/resources/TestingCredentials.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\25mee\eclipse-workspace\GroceryApplication\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\25mee\git\GroceryApplication\GroceryApplication\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04EEE49F-3575-48B3-AF09-C085BB60D0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28BB293-5FB8-4FE4-A9DD-82ABBB5B3FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPage" sheetId="1" r:id="rId1"/>
     <sheet name="AdminPage" sheetId="2" r:id="rId2"/>
-    <sheet name="ContactUsInformations" sheetId="3" r:id="rId3"/>
+    <sheet name="ContactAsInformations" sheetId="3" r:id="rId3"/>
     <sheet name="ManageNews" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
   <si>
     <t>admin</t>
   </si>
@@ -42,23 +42,20 @@
     <t>meenakshi</t>
   </si>
   <si>
-    <t>mobilenumber</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>addressfield</t>
-  </si>
-  <si>
     <t>new news headlines</t>
+  </si>
+  <si>
+    <t>test@gmail.com</t>
+  </si>
+  <si>
+    <t>adc street tvm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,6 +81,14 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -102,16 +107,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -463,10 +471,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="1">
+        <v>9133222468</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -480,6 +488,9 @@
       <c r="A3" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{2BDF1780-CB21-4D8C-934E-C83F4F19045F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -491,7 +502,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>